<commit_message>
Add required Task Type to all scheduled maintenance draft rows
</commit_message>
<xml_diff>
--- a/outputs/controls-maintenance/MHT_Controls_Maintenance_Plan.xlsx
+++ b/outputs/controls-maintenance/MHT_Controls_Maintenance_Plan.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" r:id="Rd9caf3a5d50e4a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R0f340bf5775b45fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device Register" sheetId="3" r:id="R2cf8272cb8af4f7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Map" sheetId="4" r:id="R4fb932e24f084c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" r:id="R3537b638d9c54069"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rfdb914ed06cb4a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device Register" sheetId="3" r:id="R62b3d76951eb4cd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Map" sheetId="4" r:id="Redf5640864384fc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6961,6 +6961,20 @@
         <x:v>Not published under previous source-set permission.</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="3" t="str">
+        <x:v>Task Type</x:v>
+      </x:c>
+      <x:c r="B18" s="3" t="str">
+        <x:v>User-reported tenant importer requirement</x:v>
+      </x:c>
+      <x:c r="C18" s="3" t="str">
+        <x:v>text on all 12 SM rows</x:v>
+      </x:c>
+      <x:c r="D18" s="3" t="str">
+        <x:v>Matches the data-recording task type in the task groups. Verify this field mapping in the tenant preview.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Set all controls maintenance job types to Preventative
</commit_message>
<xml_diff>
--- a/outputs/controls-maintenance/MHT_Controls_Maintenance_Plan.xlsx
+++ b/outputs/controls-maintenance/MHT_Controls_Maintenance_Plan.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" r:id="R3537b638d9c54069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rfdb914ed06cb4a04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device Register" sheetId="3" r:id="R62b3d76951eb4cd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Map" sheetId="4" r:id="Redf5640864384fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" r:id="R17e39ce62c234a06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R2f79232608ce4edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device Register" sheetId="3" r:id="R0c30dc1b752548a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Map" sheetId="4" r:id="R82dd42f16b104ff6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -298,6 +298,7 @@
     <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -331,6 +332,9 @@
       <x:c r="J1" s="5" t="str">
         <x:v>Owner - needs assignment</x:v>
       </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>Maintenance Type</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
@@ -359,6 +363,9 @@
       </x:c>
       <x:c r="I2" s="6" t="str"/>
       <x:c r="J2" s="6" t="str"/>
+      <x:c r="K2" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="3" t="str">
@@ -387,6 +394,9 @@
       </x:c>
       <x:c r="I3" s="6" t="str"/>
       <x:c r="J3" s="6" t="str"/>
+      <x:c r="K3" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="3" t="str">
@@ -415,6 +425,9 @@
       </x:c>
       <x:c r="I4" s="6" t="str"/>
       <x:c r="J4" s="6" t="str"/>
+      <x:c r="K4" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="3" t="str">
@@ -443,6 +456,9 @@
       </x:c>
       <x:c r="I5" s="6" t="str"/>
       <x:c r="J5" s="6" t="str"/>
+      <x:c r="K5" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="3" t="str">
@@ -471,6 +487,9 @@
       </x:c>
       <x:c r="I6" s="6" t="str"/>
       <x:c r="J6" s="6" t="str"/>
+      <x:c r="K6" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="3" t="str">
@@ -499,6 +518,9 @@
       </x:c>
       <x:c r="I7" s="6" t="str"/>
       <x:c r="J7" s="6" t="str"/>
+      <x:c r="K7" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="3" t="str">
@@ -527,6 +549,9 @@
       </x:c>
       <x:c r="I8" s="6" t="str"/>
       <x:c r="J8" s="6" t="str"/>
+      <x:c r="K8" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="3" t="str">
@@ -555,6 +580,9 @@
       </x:c>
       <x:c r="I9" s="6" t="str"/>
       <x:c r="J9" s="6" t="str"/>
+      <x:c r="K9" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="3" t="str">
@@ -583,6 +611,9 @@
       </x:c>
       <x:c r="I10" s="6" t="str"/>
       <x:c r="J10" s="6" t="str"/>
+      <x:c r="K10" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="3" t="str">
@@ -611,6 +642,9 @@
       </x:c>
       <x:c r="I11" s="6" t="str"/>
       <x:c r="J11" s="6" t="str"/>
+      <x:c r="K11" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="3" t="str">
@@ -639,6 +673,9 @@
       </x:c>
       <x:c r="I12" s="6" t="str"/>
       <x:c r="J12" s="6" t="str"/>
+      <x:c r="K12" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="3" t="str">
@@ -667,6 +704,9 @@
       </x:c>
       <x:c r="I13" s="6" t="str"/>
       <x:c r="J13" s="6" t="str"/>
+      <x:c r="K13" s="3" t="str">
+        <x:v>Preventative</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6975,6 +7015,20 @@
         <x:v>Matches the data-recording task type in the task groups. Verify this field mapping in the tenant preview.</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="3" t="str">
+        <x:v>Maintenance Type</x:v>
+      </x:c>
+      <x:c r="B19" s="3" t="str">
+        <x:v>User-requested job classification</x:v>
+      </x:c>
+      <x:c r="C19" s="3" t="str">
+        <x:v>Preventative on all 12 SM rows</x:v>
+      </x:c>
+      <x:c r="D19" s="3" t="str">
+        <x:v>Separate from Task Type; verify the exact tenant maintenance-type lookup.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>